<commit_message>
Aggiorna Electron Lab al 24 luglio 2026
Ricostruisce storico LL2 (91 lanci, 87 successi), agenda NET e portale con fonti Rocket Lab. Ripristina link Flight 13 su SpaceX.
</commit_message>
<xml_diff>
--- a/electronlab/lanci_electron.xlsx
+++ b/electronlab/lanci_electron.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="legenda" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'elenco'!$A$1:$P$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'elenco'!$A$1:$P$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,8 +468,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StoricoElectron" displayName="StoricoElectron" ref="A1:P91" headerRowCount="1">
-  <autoFilter ref="A1:P91"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="StoricoElectron" displayName="StoricoElectron" ref="A1:P92" headerRowCount="1">
+  <autoFilter ref="A1:P92"/>
   <tableColumns count="16">
     <tableColumn id="1" name="nr"/>
     <tableColumn id="2" name="data"/>
@@ -820,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P91"/>
+  <dimension ref="A1:P92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="N2" s="6" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=3vE2AnwJ2Qs</t>
+          <t>https://www.youtube.com/watch?v=P7YmRKuJSvU</t>
         </is>
       </c>
       <c r="O2" s="6" t="inlineStr">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Sub</t>
+          <t>LEO</t>
         </is>
       </c>
       <c r="I90" s="4" t="inlineStr"/>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="L90" s="4" t="inlineStr">
         <is>
-          <t>Sub-orbital launch under Rocket Lab’s Hypersonic Accelerator Suborbital Test Electron (HASTE) program, details TBD.</t>
+          <t>Sub-orbital launch under Rocket Lab’s Hypersonic Accelerator Suborbital Test Electron (HASTE) program, details TBD. Note: Despite reported as a strictly sub-orbital launch program, this launch was cataloged by the USSF to have left 2 rocket stages in a 200 km, 40° very low Earth orbit by the US Space Force. The payload was not cataloged and may have been deliberately de-orbited.</t>
         </is>
       </c>
       <c r="M90" s="4" t="inlineStr"/>
@@ -7203,8 +7203,80 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="3" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>17:43</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>Ten Owl Of Ten (StriX Launch 10)</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>successo</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Earth Science</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>LEO</t>
+        </is>
+      </c>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>Synspective</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Rocket Lab Launch Complex 1B</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr">
+        <is>
+          <t>Rocket Lab Launch Complex 1, Mahia Peninsula, New Zealand</t>
+        </is>
+      </c>
+      <c r="L92" s="4" t="inlineStr">
+        <is>
+          <t>Synthetic aperture radar satellite for Japanese Earth imaging company Synspective.</t>
+        </is>
+      </c>
+      <c r="M92" s="4" t="inlineStr"/>
+      <c r="N92" s="6" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=mD-rTeRXx8o</t>
+        </is>
+      </c>
+      <c r="O92" s="6" t="inlineStr">
+        <is>
+          <t>https://ll.thespacedevs.com/2.3.0/launches/add0a5be-1cf0-49cb-975a-e8c8e18d37ec/?format=json</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>add0a5be-1cf0-49cb-975a-e8c8e18d37ec</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P91"/>
+  <autoFilter ref="A1:P92"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId2"/>
@@ -7380,10 +7452,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O90" r:id="rId172"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N91" r:id="rId173"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O91" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N92" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O92" r:id="rId176"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId175"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId177"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7419,7 +7493,7 @@
     <row r="2" ht="23" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Dati aggiornati al 24/06/2026 07:48 · Fonte: The Space Devs / Launch Library 2</t>
+          <t>Dati aggiornati al 24/07/2026 12:03 · Fonte: The Space Devs / Launch Library 2</t>
         </is>
       </c>
     </row>
@@ -7447,16 +7521,16 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>4</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>0.9555555555555556</v>
+        <v>0.9560439560439561</v>
       </c>
     </row>
     <row r="7">
@@ -7486,10 +7560,10 @@
         <v>42880</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>46192</v>
+        <v>46199</v>
       </c>
       <c r="E8" s="11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G8" s="11" t="n">
         <v>3</v>
@@ -7503,7 +7577,7 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>#90 · VICTUS HAZE Puma · 19/06/2026</t>
+          <t>#91 · Ten Owl Of Ten (StriX Launch 10) · 26/06/2026</t>
         </is>
       </c>
     </row>
@@ -7764,10 +7838,10 @@
         <v>2026</v>
       </c>
       <c r="B14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -7850,7 +7924,7 @@
         <v>41</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>0.4555555555555555</v>
+        <v>0.4505494505494506</v>
       </c>
       <c r="D5" s="17" t="n">
         <v>46192</v>
@@ -7863,13 +7937,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.4</v>
+        <v>0.4065934065934066</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>46164</v>
+        <v>46199</v>
       </c>
     </row>
     <row r="7">
@@ -7882,7 +7956,7 @@
         <v>13</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>0.1444444444444444</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="D7" s="17" t="n">
         <v>46184</v>
@@ -7952,10 +8026,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>0.5</v>
+        <v>0.5164835164835165</v>
       </c>
     </row>
     <row r="6">
@@ -7968,7 +8042,7 @@
         <v>31</v>
       </c>
       <c r="C6" s="16" t="n">
-        <v>0.3444444444444444</v>
+        <v>0.3406593406593407</v>
       </c>
     </row>
     <row r="7">
@@ -7978,10 +8052,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>0.1</v>
+        <v>0.08791208791208792</v>
       </c>
     </row>
     <row r="8">
@@ -7994,7 +8068,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="16" t="n">
-        <v>0.04444444444444445</v>
+        <v>0.04395604395604396</v>
       </c>
     </row>
     <row r="9">
@@ -8007,7 +8081,7 @@
         <v>1</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>0.01111111111111111</v>
+        <v>0.01098901098901099</v>
       </c>
     </row>
   </sheetData>

</xml_diff>